<commit_message>
feat: align dimensional properties and visual scaling for wellbore database
- Update valor_free1.py to correctly structure the 3-phase casing and hole sections as per Excel spec.

- Refactor fancy_well_database.py to compute sheaf dimensions and scale visual lengths accurately.

- Enhance Excel automation in create_wellbore_excel.py for detailed WBD representations.

- Generate K_S_evidence and frozen_snapshot JSONs for closure.
</commit_message>
<xml_diff>
--- a/artifacts/Wellbore_Diagram_State_Free1.xlsx
+++ b/artifacts/Wellbore_Diagram_State_Free1.xlsx
@@ -110,7 +110,7 @@
       <sz val="9"/>
     </font>
   </fonts>
-  <fills count="11">
+  <fills count="12">
     <fill>
       <patternFill/>
     </fill>
@@ -157,6 +157,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="0015803d"/>
         <bgColor rgb="0015803d"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00475569"/>
+        <bgColor rgb="00475569"/>
       </patternFill>
     </fill>
     <fill>
@@ -212,7 +218,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="36">
+  <cellXfs count="41">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -262,13 +268,20 @@
     <xf numFmtId="0" fontId="6" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="9" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="9" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="10" fillId="9" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="10" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
@@ -286,9 +299,13 @@
     </xf>
     <xf numFmtId="0" fontId="13" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="13" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="14" fillId="9" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="15" fillId="10" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="16" fillId="10" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="14" fillId="10" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="15" fillId="11" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="16" fillId="11" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -654,7 +671,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I26"/>
+  <dimension ref="A1:I27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -864,17 +881,15 @@
       <c r="C16" s="14" t="n">
         <v>13.375</v>
       </c>
-      <c r="D16" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="D16" s="14" t="n">
+        <v>12.615</v>
       </c>
       <c r="E16" s="14" t="n">
         <v>54</v>
       </c>
       <c r="F16" s="14" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>J-55 / 8rd</t>
         </is>
       </c>
       <c r="G16" s="14" t="n">
@@ -882,7 +897,7 @@
       </c>
       <c r="H16" s="14" t="inlineStr">
         <is>
-          <t>125.0 / 15.7 Spud Mud (Lead/Tail)</t>
+          <t>125.0 / 15.7 Spud Mud</t>
         </is>
       </c>
       <c r="I16" s="14" t="n">
@@ -899,13 +914,13 @@
         <v>12.25</v>
       </c>
       <c r="C17" s="16" t="n">
-        <v>13.375</v>
+        <v>7</v>
       </c>
       <c r="D17" s="16" t="n">
-        <v>12.615</v>
+        <v>6.366</v>
       </c>
       <c r="E17" s="16" t="n">
-        <v>54</v>
+        <v>23</v>
       </c>
       <c r="F17" s="16" t="inlineStr">
         <is>
@@ -917,59 +932,94 @@
       </c>
       <c r="H17" s="16" t="inlineStr">
         <is>
-          <t>- / -</t>
-        </is>
-      </c>
-      <c r="I17" s="16" t="inlineStr">
+          <t>266.0 / 15.7 Spud Mud</t>
+        </is>
+      </c>
+      <c r="I17" s="16" t="n">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="17" t="inlineStr">
+        <is>
+          <t>Production</t>
+        </is>
+      </c>
+      <c r="B18" s="18" t="n">
+        <v>6</v>
+      </c>
+      <c r="C18" s="18" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="D18" s="18" t="n">
+        <v>3.875</v>
+      </c>
+      <c r="E18" s="18" t="n">
+        <v>11.6</v>
+      </c>
+      <c r="F18" s="18" t="inlineStr">
+        <is>
+          <t>L-80 / 8rd</t>
+        </is>
+      </c>
+      <c r="G18" s="18" t="n">
+        <v>2000</v>
+      </c>
+      <c r="H18" s="18" t="inlineStr">
+        <is>
+          <t>765.0 / 14.8 Air Drill</t>
+        </is>
+      </c>
+      <c r="I18" s="18" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="17" t="inlineStr">
+    <row r="21">
+      <c r="A21" s="19" t="inlineStr">
         <is>
           <t>NOTES &amp; PROVENANCE</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="18" t="inlineStr">
+    <row r="22">
+      <c r="A22" s="20" t="inlineStr">
         <is>
           <t>• Data source: Research documents (Action Plan + OBJECT-PLAN-CONCEPT PDFs) + welly_db_4budZ harness (FancyWellDatabaseObject).</t>
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="18" t="inlineStr">
+    <row r="23">
+      <c r="A23" s="20" t="inlineStr">
         <is>
           <t>• This file is a native .xlsx realization of the 'spreadsheet of excellence' concept with visual schematic.</t>
         </is>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" s="18" t="inlineStr">
+    <row r="24">
+      <c r="A24" s="20" t="inlineStr">
         <is>
           <t>• Topological verification (from harness run): Δλ₁ ≈ +0.080 (positive coherence harvest), holonomy trivial on baseline seed.</t>
         </is>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" s="18" t="inlineStr">
+    <row r="25">
+      <c r="A25" s="20" t="inlineStr">
         <is>
           <t>• For directional/horizontal wells: add columns for Inclination, Azimuth, TVD, and adjust schematic accordingly.</t>
         </is>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" s="18" t="inlineStr">
+    <row r="26">
+      <c r="A26" s="20" t="inlineStr">
         <is>
           <t>• Deeper casing strings (Intermediate 7", Production 4.5") from original Eric Excel can be appended to the tables above.</t>
         </is>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" s="18" t="inlineStr">
+    <row r="27">
+      <c r="A27" s="20" t="inlineStr">
         <is>
           <t>• Do not edit depths/diameters without re-running the welly_db harness for new K(S) evidence.</t>
         </is>
@@ -985,9 +1035,9 @@
     <mergeCell ref="A2:H2"/>
     <mergeCell ref="A14:I14"/>
     <mergeCell ref="A23:I23"/>
+    <mergeCell ref="A27:I27"/>
+    <mergeCell ref="A1:H1"/>
     <mergeCell ref="A24:I24"/>
-    <mergeCell ref="A1:H1"/>
-    <mergeCell ref="A20:I20"/>
     <mergeCell ref="A21:I21"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1000,14 +1050,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F51"/>
+  <dimension ref="A1:F136"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="18" customWidth="1" min="2" max="2"/>
     <col width="22" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="32" customWidth="1" min="5" max="5"/>
+    <col width="64" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1" ht="26" customHeight="1">
@@ -1020,629 +1070,1649 @@
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>Vertical scale approximate (1 row ≈ 10 ft). Not to horizontal scale. Colors per research regimes (Stable=green, Transitional=yellow/olive).</t>
+          <t>Vertical scale approximate (1 row = 20 ft). Not to horizontal scale. Colors per research regimes (Stable=green, Transitional=yellow/olive).</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="19" t="inlineStr">
+      <c r="A4" s="21" t="inlineStr">
         <is>
           <t>LEGEND:</t>
         </is>
       </c>
-      <c r="B4" s="20" t="inlineStr">
+      <c r="B4" s="22" t="inlineStr">
         <is>
           <t>Conductor</t>
         </is>
       </c>
-      <c r="C4" s="21" t="inlineStr">
+      <c r="C4" s="23" t="inlineStr">
         <is>
           <t>Surface Csg</t>
         </is>
       </c>
-      <c r="D4" s="22" t="inlineStr">
+      <c r="D4" s="24" t="inlineStr">
+        <is>
+          <t>Production Csg</t>
+        </is>
+      </c>
+      <c r="E4" s="25" t="inlineStr">
         <is>
           <t>Formation / Rock</t>
         </is>
       </c>
-      <c r="E4" s="23" t="inlineStr">
+      <c r="F4" s="26" t="inlineStr">
         <is>
           <t>Open Hole / Mud</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="24" t="inlineStr">
+      <c r="A6" s="27" t="inlineStr">
         <is>
           <t>Depth (ft)</t>
         </is>
       </c>
-      <c r="B6" s="24" t="inlineStr">
+      <c r="B6" s="27" t="inlineStr">
         <is>
           <t>Formation</t>
         </is>
       </c>
-      <c r="C6" s="24" t="inlineStr">
+      <c r="C6" s="27" t="inlineStr">
         <is>
           <t>Schematic (Casing / Hole)</t>
         </is>
       </c>
-      <c r="D6" s="24" t="inlineStr">
+      <c r="D6" s="27" t="inlineStr">
         <is>
           <t>Casing OD</t>
         </is>
       </c>
-      <c r="E6" s="24" t="inlineStr">
+      <c r="E6" s="27" t="inlineStr">
         <is>
           <t>Notes / Cement</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="25" t="n">
+      <c r="A7" s="28" t="n">
         <v>0</v>
       </c>
-      <c r="B7" s="26" t="n"/>
-      <c r="C7" s="27" t="inlineStr">
+      <c r="B7" s="29" t="n"/>
+      <c r="C7" s="30" t="inlineStr">
         <is>
           <t xml:space="preserve">  13.375"  </t>
         </is>
       </c>
-      <c r="D7" s="28" t="inlineStr">
+      <c r="D7" s="31" t="inlineStr">
         <is>
           <t>13.375" Cond</t>
         </is>
       </c>
-      <c r="E7" s="29" t="inlineStr">
-        <is>
-          <t>17.5" hole • 125 sks 15.7ppg Spud • WOB 15k</t>
-        </is>
-      </c>
+      <c r="E7" s="29" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="25" t="inlineStr"/>
-      <c r="B8" s="26" t="n"/>
-      <c r="C8" s="27" t="inlineStr"/>
-      <c r="D8" s="26" t="n"/>
-      <c r="E8" s="29" t="inlineStr">
-        <is>
-          <t>17.5" hole • 125 sks 15.7ppg Spud • WOB 15k</t>
+      <c r="A8" s="28" t="inlineStr"/>
+      <c r="B8" s="29" t="n"/>
+      <c r="C8" s="30" t="inlineStr"/>
+      <c r="D8" s="29" t="n"/>
+      <c r="E8" s="32" t="inlineStr">
+        <is>
+          <t>Hole: 17.5" • CSG: 13.375" OD, 12.615" ID, J-55 54# • Cement: 125 sks 15.7ppg Spud • WOB 15k, ROP 100</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="25" t="n">
-        <v>20</v>
-      </c>
-      <c r="B9" s="26" t="n"/>
-      <c r="C9" s="27" t="inlineStr">
+      <c r="A9" s="28" t="n">
+        <v>40</v>
+      </c>
+      <c r="B9" s="29" t="n"/>
+      <c r="C9" s="30" t="inlineStr">
         <is>
           <t xml:space="preserve">  13.375"  </t>
         </is>
       </c>
-      <c r="D9" s="28" t="inlineStr">
+      <c r="D9" s="31" t="inlineStr">
         <is>
           <t>13.375" Cond</t>
         </is>
       </c>
-      <c r="E9" s="26" t="n"/>
+      <c r="E9" s="29" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="25" t="inlineStr"/>
-      <c r="B10" s="26" t="n"/>
-      <c r="C10" s="27" t="inlineStr"/>
-      <c r="D10" s="26" t="n"/>
-      <c r="E10" s="26" t="n"/>
+      <c r="A10" s="28" t="inlineStr"/>
+      <c r="B10" s="29" t="n"/>
+      <c r="C10" s="30" t="inlineStr"/>
+      <c r="D10" s="29" t="n"/>
+      <c r="E10" s="29" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="25" t="n">
-        <v>40</v>
-      </c>
-      <c r="B11" s="26" t="n"/>
-      <c r="C11" s="27" t="inlineStr">
+      <c r="A11" s="28" t="n">
+        <v>80</v>
+      </c>
+      <c r="B11" s="29" t="n"/>
+      <c r="C11" s="30" t="inlineStr">
         <is>
           <t xml:space="preserve">  13.375"  </t>
         </is>
       </c>
-      <c r="D11" s="28" t="inlineStr">
+      <c r="D11" s="31" t="inlineStr">
         <is>
           <t>13.375" Cond</t>
         </is>
       </c>
-      <c r="E11" s="26" t="n"/>
+      <c r="E11" s="29" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="25" t="inlineStr"/>
-      <c r="B12" s="26" t="n"/>
-      <c r="C12" s="27" t="inlineStr"/>
-      <c r="D12" s="26" t="n"/>
-      <c r="E12" s="26" t="n"/>
+      <c r="A12" s="28" t="inlineStr"/>
+      <c r="B12" s="29" t="n"/>
+      <c r="C12" s="30" t="inlineStr"/>
+      <c r="D12" s="29" t="n"/>
+      <c r="E12" s="29" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="25" t="n">
-        <v>60</v>
-      </c>
-      <c r="B13" s="26" t="n"/>
-      <c r="C13" s="27" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  13.375"  </t>
-        </is>
-      </c>
-      <c r="D13" s="28" t="inlineStr">
-        <is>
-          <t>13.375" Cond</t>
-        </is>
-      </c>
-      <c r="E13" s="26" t="n"/>
+      <c r="A13" s="28" t="n">
+        <v>120</v>
+      </c>
+      <c r="B13" s="29" t="n"/>
+      <c r="C13" s="33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  7.0"  </t>
+        </is>
+      </c>
+      <c r="D13" s="31" t="inlineStr">
+        <is>
+          <t>7.0" Surf</t>
+        </is>
+      </c>
+      <c r="E13" s="29" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="25" t="inlineStr"/>
-      <c r="B14" s="26" t="n"/>
-      <c r="C14" s="27" t="inlineStr"/>
-      <c r="D14" s="26" t="n"/>
-      <c r="E14" s="26" t="n"/>
+      <c r="A14" s="28" t="inlineStr"/>
+      <c r="B14" s="34" t="inlineStr">
+        <is>
+          <t>Ohio Shale</t>
+        </is>
+      </c>
+      <c r="C14" s="33" t="inlineStr"/>
+      <c r="D14" s="29" t="n"/>
+      <c r="E14" s="32" t="inlineStr">
+        <is>
+          <t>Hole: 12.25" • CSG: 7" OD, 6.366" ID, J-55 23# • Cement: 266 sks 15.7ppg Spud • WOB 25k, ROP 150</t>
+        </is>
+      </c>
     </row>
     <row r="15">
-      <c r="A15" s="25" t="n">
-        <v>80</v>
-      </c>
-      <c r="B15" s="26" t="n"/>
-      <c r="C15" s="27" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  13.375"  </t>
-        </is>
-      </c>
-      <c r="D15" s="28" t="inlineStr">
-        <is>
-          <t>13.375" Cond</t>
-        </is>
-      </c>
-      <c r="E15" s="26" t="n"/>
+      <c r="A15" s="28" t="n">
+        <v>160</v>
+      </c>
+      <c r="B15" s="34" t="inlineStr"/>
+      <c r="C15" s="33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  7.0"  </t>
+        </is>
+      </c>
+      <c r="D15" s="31" t="inlineStr">
+        <is>
+          <t>7.0" Surf</t>
+        </is>
+      </c>
+      <c r="E15" s="29" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="25" t="inlineStr"/>
-      <c r="B16" s="26" t="n"/>
-      <c r="C16" s="27" t="inlineStr"/>
-      <c r="D16" s="26" t="n"/>
-      <c r="E16" s="26" t="n"/>
+      <c r="A16" s="28" t="inlineStr"/>
+      <c r="B16" s="34" t="inlineStr">
+        <is>
+          <t>Ohio Shale</t>
+        </is>
+      </c>
+      <c r="C16" s="33" t="inlineStr"/>
+      <c r="D16" s="29" t="n"/>
+      <c r="E16" s="29" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" s="25" t="n">
-        <v>100</v>
-      </c>
-      <c r="B17" s="26" t="n"/>
-      <c r="C17" s="27" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  13.375"  </t>
-        </is>
-      </c>
-      <c r="D17" s="28" t="inlineStr">
-        <is>
-          <t>13.375" Cond</t>
-        </is>
-      </c>
-      <c r="E17" s="26" t="n"/>
+      <c r="A17" s="28" t="n">
+        <v>200</v>
+      </c>
+      <c r="B17" s="34" t="inlineStr"/>
+      <c r="C17" s="33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  7.0"  </t>
+        </is>
+      </c>
+      <c r="D17" s="31" t="inlineStr">
+        <is>
+          <t>7.0" Surf</t>
+        </is>
+      </c>
+      <c r="E17" s="29" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="25" t="inlineStr"/>
-      <c r="B18" s="26" t="n"/>
-      <c r="C18" s="27" t="inlineStr"/>
-      <c r="D18" s="26" t="n"/>
-      <c r="E18" s="26" t="n"/>
+      <c r="A18" s="28" t="inlineStr"/>
+      <c r="B18" s="34" t="inlineStr"/>
+      <c r="C18" s="33" t="inlineStr"/>
+      <c r="D18" s="29" t="n"/>
+      <c r="E18" s="29" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="25" t="n">
-        <v>120</v>
-      </c>
-      <c r="B19" s="26" t="n"/>
-      <c r="C19" s="30" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  13.375"  </t>
-        </is>
-      </c>
-      <c r="D19" s="28" t="inlineStr">
-        <is>
-          <t>13.375" Surf</t>
-        </is>
-      </c>
-      <c r="E19" s="26" t="n"/>
+      <c r="A19" s="28" t="n">
+        <v>240</v>
+      </c>
+      <c r="B19" s="34" t="inlineStr">
+        <is>
+          <t>Ohio Shale</t>
+        </is>
+      </c>
+      <c r="C19" s="33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  7.0"  </t>
+        </is>
+      </c>
+      <c r="D19" s="31" t="inlineStr">
+        <is>
+          <t>7.0" Surf</t>
+        </is>
+      </c>
+      <c r="E19" s="29" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" s="25" t="inlineStr"/>
-      <c r="B20" s="31" t="inlineStr">
-        <is>
-          <t>Ohio Shale</t>
-        </is>
-      </c>
-      <c r="C20" s="30" t="inlineStr"/>
-      <c r="D20" s="26" t="n"/>
-      <c r="E20" s="26" t="n"/>
+      <c r="A20" s="28" t="inlineStr"/>
+      <c r="B20" s="34" t="inlineStr"/>
+      <c r="C20" s="33" t="inlineStr"/>
+      <c r="D20" s="29" t="n"/>
+      <c r="E20" s="29" t="n"/>
     </row>
     <row r="21">
-      <c r="A21" s="25" t="n">
-        <v>140</v>
-      </c>
-      <c r="B21" s="31" t="inlineStr">
-        <is>
-          <t>Ohio Shale</t>
-        </is>
-      </c>
-      <c r="C21" s="30" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  13.375"  </t>
-        </is>
-      </c>
-      <c r="D21" s="28" t="inlineStr">
-        <is>
-          <t>13.375" Surf</t>
-        </is>
-      </c>
-      <c r="E21" s="26" t="n"/>
+      <c r="A21" s="28" t="n">
+        <v>280</v>
+      </c>
+      <c r="B21" s="35" t="inlineStr">
+        <is>
+          <t>Big Lime</t>
+        </is>
+      </c>
+      <c r="C21" s="33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  7.0"  </t>
+        </is>
+      </c>
+      <c r="D21" s="31" t="inlineStr">
+        <is>
+          <t>7.0" Surf</t>
+        </is>
+      </c>
+      <c r="E21" s="29" t="n"/>
     </row>
     <row r="22">
-      <c r="A22" s="25" t="inlineStr"/>
-      <c r="B22" s="31" t="inlineStr">
-        <is>
-          <t>Ohio Shale</t>
-        </is>
-      </c>
-      <c r="C22" s="30" t="inlineStr"/>
-      <c r="D22" s="26" t="n"/>
-      <c r="E22" s="26" t="n"/>
+      <c r="A22" s="28" t="inlineStr"/>
+      <c r="B22" s="35" t="inlineStr">
+        <is>
+          <t>Big Lime</t>
+        </is>
+      </c>
+      <c r="C22" s="33" t="inlineStr"/>
+      <c r="D22" s="29" t="n"/>
+      <c r="E22" s="29" t="n"/>
     </row>
     <row r="23">
-      <c r="A23" s="25" t="n">
-        <v>160</v>
-      </c>
-      <c r="B23" s="31" t="inlineStr"/>
-      <c r="C23" s="30" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  13.375"  </t>
-        </is>
-      </c>
-      <c r="D23" s="28" t="inlineStr">
-        <is>
-          <t>13.375" Surf</t>
-        </is>
-      </c>
-      <c r="E23" s="26" t="n"/>
+      <c r="A23" s="28" t="n">
+        <v>320</v>
+      </c>
+      <c r="B23" s="35" t="inlineStr"/>
+      <c r="C23" s="33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  7.0"  </t>
+        </is>
+      </c>
+      <c r="D23" s="31" t="inlineStr">
+        <is>
+          <t>7.0" Surf</t>
+        </is>
+      </c>
+      <c r="E23" s="29" t="n"/>
     </row>
     <row r="24">
-      <c r="A24" s="25" t="inlineStr"/>
-      <c r="B24" s="31" t="inlineStr"/>
-      <c r="C24" s="30" t="inlineStr"/>
-      <c r="D24" s="26" t="n"/>
-      <c r="E24" s="26" t="n"/>
+      <c r="A24" s="28" t="inlineStr"/>
+      <c r="B24" s="35" t="inlineStr"/>
+      <c r="C24" s="33" t="inlineStr"/>
+      <c r="D24" s="29" t="n"/>
+      <c r="E24" s="29" t="n"/>
     </row>
     <row r="25">
-      <c r="A25" s="25" t="n">
-        <v>180</v>
-      </c>
-      <c r="B25" s="31" t="inlineStr">
-        <is>
-          <t>Ohio Shale</t>
-        </is>
-      </c>
-      <c r="C25" s="30" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  13.375"  </t>
-        </is>
-      </c>
-      <c r="D25" s="28" t="inlineStr">
-        <is>
-          <t>13.375" Surf</t>
-        </is>
-      </c>
-      <c r="E25" s="26" t="n"/>
+      <c r="A25" s="28" t="n">
+        <v>360</v>
+      </c>
+      <c r="B25" s="35" t="inlineStr">
+        <is>
+          <t>Big Lime</t>
+        </is>
+      </c>
+      <c r="C25" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  4.5"  </t>
+        </is>
+      </c>
+      <c r="D25" s="31" t="inlineStr">
+        <is>
+          <t>4.5" Prod</t>
+        </is>
+      </c>
+      <c r="E25" s="29" t="n"/>
     </row>
     <row r="26">
-      <c r="A26" s="25" t="inlineStr"/>
-      <c r="B26" s="31" t="inlineStr"/>
-      <c r="C26" s="30" t="inlineStr"/>
-      <c r="D26" s="26" t="n"/>
-      <c r="E26" s="26" t="n"/>
+      <c r="A26" s="28" t="inlineStr"/>
+      <c r="B26" s="35" t="inlineStr"/>
+      <c r="C26" s="36" t="inlineStr"/>
+      <c r="D26" s="29" t="n"/>
+      <c r="E26" s="32" t="inlineStr">
+        <is>
+          <t>Hole: 6" • CSG: 4.5" OD, 3.875" ID, L-80 11.6# • Cement: 765 sks 12-14.8ppg Air • WOB XX, ROP XX</t>
+        </is>
+      </c>
     </row>
     <row r="27">
-      <c r="A27" s="25" t="n">
-        <v>200</v>
-      </c>
-      <c r="B27" s="31" t="inlineStr"/>
-      <c r="C27" s="30" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  13.375"  </t>
-        </is>
-      </c>
-      <c r="D27" s="28" t="inlineStr">
-        <is>
-          <t>13.375" Surf</t>
-        </is>
-      </c>
-      <c r="E27" s="26" t="n"/>
+      <c r="A27" s="28" t="n">
+        <v>400</v>
+      </c>
+      <c r="B27" s="35" t="inlineStr"/>
+      <c r="C27" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  4.5"  </t>
+        </is>
+      </c>
+      <c r="D27" s="31" t="inlineStr">
+        <is>
+          <t>4.5" Prod</t>
+        </is>
+      </c>
+      <c r="E27" s="29" t="n"/>
     </row>
     <row r="28">
-      <c r="A28" s="25" t="inlineStr"/>
-      <c r="B28" s="31" t="inlineStr">
-        <is>
-          <t>Ohio Shale</t>
-        </is>
-      </c>
-      <c r="C28" s="30" t="inlineStr"/>
-      <c r="D28" s="26" t="n"/>
-      <c r="E28" s="26" t="n"/>
+      <c r="A28" s="28" t="inlineStr"/>
+      <c r="B28" s="35" t="inlineStr">
+        <is>
+          <t>Big Lime</t>
+        </is>
+      </c>
+      <c r="C28" s="36" t="inlineStr"/>
+      <c r="D28" s="29" t="n"/>
+      <c r="E28" s="29" t="n"/>
     </row>
     <row r="29">
-      <c r="A29" s="25" t="n">
-        <v>220</v>
-      </c>
-      <c r="B29" s="31" t="inlineStr"/>
-      <c r="C29" s="30" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  13.375"  </t>
-        </is>
-      </c>
-      <c r="D29" s="28" t="inlineStr">
-        <is>
-          <t>13.375" Surf</t>
-        </is>
-      </c>
-      <c r="E29" s="26" t="n"/>
+      <c r="A29" s="28" t="n">
+        <v>440</v>
+      </c>
+      <c r="B29" s="35" t="inlineStr"/>
+      <c r="C29" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  4.5"  </t>
+        </is>
+      </c>
+      <c r="D29" s="31" t="inlineStr">
+        <is>
+          <t>4.5" Prod</t>
+        </is>
+      </c>
+      <c r="E29" s="29" t="n"/>
     </row>
     <row r="30">
-      <c r="A30" s="25" t="inlineStr"/>
-      <c r="B30" s="31" t="inlineStr"/>
-      <c r="C30" s="30" t="inlineStr"/>
-      <c r="D30" s="26" t="n"/>
-      <c r="E30" s="26" t="n"/>
+      <c r="A30" s="28" t="inlineStr"/>
+      <c r="B30" s="35" t="inlineStr"/>
+      <c r="C30" s="36" t="inlineStr"/>
+      <c r="D30" s="29" t="n"/>
+      <c r="E30" s="29" t="n"/>
     </row>
     <row r="31">
-      <c r="A31" s="25" t="n">
-        <v>240</v>
-      </c>
-      <c r="B31" s="31" t="inlineStr">
-        <is>
-          <t>Ohio Shale</t>
-        </is>
-      </c>
-      <c r="C31" s="30" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  13.375"  </t>
-        </is>
-      </c>
-      <c r="D31" s="28" t="inlineStr">
-        <is>
-          <t>13.375" Surf</t>
-        </is>
-      </c>
-      <c r="E31" s="26" t="n"/>
+      <c r="A31" s="28" t="n">
+        <v>480</v>
+      </c>
+      <c r="B31" s="35" t="inlineStr">
+        <is>
+          <t>Big Lime</t>
+        </is>
+      </c>
+      <c r="C31" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  4.5"  </t>
+        </is>
+      </c>
+      <c r="D31" s="31" t="inlineStr">
+        <is>
+          <t>4.5" Prod</t>
+        </is>
+      </c>
+      <c r="E31" s="29" t="n"/>
     </row>
     <row r="32">
-      <c r="A32" s="25" t="inlineStr"/>
-      <c r="B32" s="31" t="inlineStr"/>
-      <c r="C32" s="30" t="inlineStr"/>
-      <c r="D32" s="26" t="n"/>
-      <c r="E32" s="26" t="n"/>
+      <c r="A32" s="28" t="inlineStr"/>
+      <c r="B32" s="35" t="inlineStr"/>
+      <c r="C32" s="36" t="inlineStr"/>
+      <c r="D32" s="29" t="n"/>
+      <c r="E32" s="29" t="n"/>
     </row>
     <row r="33">
-      <c r="A33" s="25" t="n">
-        <v>260</v>
-      </c>
-      <c r="B33" s="31" t="inlineStr"/>
-      <c r="C33" s="30" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  13.375"  </t>
-        </is>
-      </c>
-      <c r="D33" s="28" t="inlineStr">
-        <is>
-          <t>13.375" Surf</t>
-        </is>
-      </c>
-      <c r="E33" s="26" t="n"/>
+      <c r="A33" s="28" t="n">
+        <v>520</v>
+      </c>
+      <c r="B33" s="35" t="inlineStr"/>
+      <c r="C33" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  4.5"  </t>
+        </is>
+      </c>
+      <c r="D33" s="31" t="inlineStr">
+        <is>
+          <t>4.5" Prod</t>
+        </is>
+      </c>
+      <c r="E33" s="29" t="n"/>
     </row>
     <row r="34">
-      <c r="A34" s="25" t="inlineStr"/>
-      <c r="B34" s="32" t="inlineStr">
+      <c r="A34" s="28" t="inlineStr"/>
+      <c r="B34" s="35" t="inlineStr">
         <is>
           <t>Big Lime</t>
         </is>
       </c>
-      <c r="C34" s="30" t="inlineStr"/>
-      <c r="D34" s="26" t="n"/>
-      <c r="E34" s="26" t="n"/>
+      <c r="C34" s="36" t="inlineStr"/>
+      <c r="D34" s="29" t="n"/>
+      <c r="E34" s="29" t="n"/>
     </row>
     <row r="35">
-      <c r="A35" s="25" t="n">
-        <v>280</v>
-      </c>
-      <c r="B35" s="32" t="inlineStr">
+      <c r="A35" s="28" t="n">
+        <v>560</v>
+      </c>
+      <c r="B35" s="35" t="inlineStr"/>
+      <c r="C35" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  4.5"  </t>
+        </is>
+      </c>
+      <c r="D35" s="31" t="inlineStr">
+        <is>
+          <t>4.5" Prod</t>
+        </is>
+      </c>
+      <c r="E35" s="29" t="n"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="28" t="inlineStr"/>
+      <c r="B36" s="35" t="inlineStr"/>
+      <c r="C36" s="36" t="inlineStr"/>
+      <c r="D36" s="29" t="n"/>
+      <c r="E36" s="29" t="n"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="28" t="n">
+        <v>600</v>
+      </c>
+      <c r="B37" s="35" t="inlineStr">
         <is>
           <t>Big Lime</t>
         </is>
       </c>
-      <c r="C35" s="30" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  13.375"  </t>
-        </is>
-      </c>
-      <c r="D35" s="28" t="inlineStr">
-        <is>
-          <t>13.375" Surf</t>
-        </is>
-      </c>
-      <c r="E35" s="26" t="n"/>
-    </row>
-    <row r="36">
-      <c r="A36" s="25" t="inlineStr"/>
-      <c r="B36" s="32" t="inlineStr"/>
-      <c r="C36" s="30" t="inlineStr"/>
-      <c r="D36" s="26" t="n"/>
-      <c r="E36" s="26" t="n"/>
-    </row>
-    <row r="37">
-      <c r="A37" s="25" t="n">
-        <v>300</v>
-      </c>
-      <c r="B37" s="32" t="inlineStr">
+      <c r="C37" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  4.5"  </t>
+        </is>
+      </c>
+      <c r="D37" s="31" t="inlineStr">
+        <is>
+          <t>4.5" Prod</t>
+        </is>
+      </c>
+      <c r="E37" s="29" t="n"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="28" t="inlineStr"/>
+      <c r="B38" s="35" t="inlineStr"/>
+      <c r="C38" s="36" t="inlineStr"/>
+      <c r="D38" s="29" t="n"/>
+      <c r="E38" s="29" t="n"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="28" t="n">
+        <v>640</v>
+      </c>
+      <c r="B39" s="35" t="inlineStr"/>
+      <c r="C39" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  4.5"  </t>
+        </is>
+      </c>
+      <c r="D39" s="31" t="inlineStr">
+        <is>
+          <t>4.5" Prod</t>
+        </is>
+      </c>
+      <c r="E39" s="29" t="n"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="28" t="inlineStr"/>
+      <c r="B40" s="35" t="inlineStr">
         <is>
           <t>Big Lime</t>
         </is>
       </c>
-      <c r="C37" s="30" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  13.375"  </t>
-        </is>
-      </c>
-      <c r="D37" s="28" t="inlineStr">
-        <is>
-          <t>13.375" Surf</t>
-        </is>
-      </c>
-      <c r="E37" s="26" t="n"/>
-    </row>
-    <row r="38">
-      <c r="A38" s="25" t="inlineStr"/>
-      <c r="B38" s="32" t="inlineStr"/>
-      <c r="C38" s="30" t="inlineStr"/>
-      <c r="D38" s="26" t="n"/>
-      <c r="E38" s="26" t="n"/>
-    </row>
-    <row r="39">
-      <c r="A39" s="25" t="n">
-        <v>320</v>
-      </c>
-      <c r="B39" s="32" t="inlineStr"/>
-      <c r="C39" s="30" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  13.375"  </t>
-        </is>
-      </c>
-      <c r="D39" s="28" t="inlineStr">
-        <is>
-          <t>13.375" Surf</t>
-        </is>
-      </c>
-      <c r="E39" s="26" t="n"/>
-    </row>
-    <row r="40">
-      <c r="A40" s="25" t="inlineStr"/>
-      <c r="B40" s="32" t="inlineStr">
-        <is>
-          <t>Big Lime</t>
-        </is>
-      </c>
-      <c r="C40" s="30" t="inlineStr"/>
-      <c r="D40" s="26" t="n"/>
-      <c r="E40" s="26" t="n"/>
+      <c r="C40" s="36" t="inlineStr"/>
+      <c r="D40" s="29" t="n"/>
+      <c r="E40" s="29" t="n"/>
     </row>
     <row r="41">
-      <c r="A41" s="25" t="n">
-        <v>340</v>
-      </c>
-      <c r="B41" s="32" t="inlineStr"/>
-      <c r="C41" s="30" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  13.375"  </t>
-        </is>
-      </c>
-      <c r="D41" s="28" t="inlineStr">
-        <is>
-          <t>13.375" Surf</t>
-        </is>
-      </c>
-      <c r="E41" s="26" t="n"/>
+      <c r="A41" s="28" t="n">
+        <v>680</v>
+      </c>
+      <c r="B41" s="35" t="inlineStr"/>
+      <c r="C41" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  4.5"  </t>
+        </is>
+      </c>
+      <c r="D41" s="31" t="inlineStr">
+        <is>
+          <t>4.5" Prod</t>
+        </is>
+      </c>
+      <c r="E41" s="29" t="n"/>
     </row>
     <row r="42">
-      <c r="A42" s="25" t="inlineStr"/>
-      <c r="B42" s="32" t="inlineStr"/>
-      <c r="C42" s="30" t="inlineStr"/>
-      <c r="D42" s="26" t="n"/>
-      <c r="E42" s="26" t="n"/>
+      <c r="A42" s="28" t="inlineStr"/>
+      <c r="B42" s="35" t="inlineStr"/>
+      <c r="C42" s="36" t="inlineStr"/>
+      <c r="D42" s="29" t="n"/>
+      <c r="E42" s="29" t="n"/>
     </row>
     <row r="43">
-      <c r="A43" s="25" t="n">
-        <v>360</v>
-      </c>
-      <c r="B43" s="32" t="inlineStr">
-        <is>
-          <t>Big Lime</t>
-        </is>
-      </c>
-      <c r="C43" s="33" t="inlineStr">
+      <c r="A43" s="28" t="n">
+        <v>720</v>
+      </c>
+      <c r="B43" s="29" t="n"/>
+      <c r="C43" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  4.5"  </t>
+        </is>
+      </c>
+      <c r="D43" s="31" t="inlineStr">
+        <is>
+          <t>4.5" Prod</t>
+        </is>
+      </c>
+      <c r="E43" s="29" t="n"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="28" t="inlineStr"/>
+      <c r="B44" s="29" t="n"/>
+      <c r="C44" s="36" t="inlineStr"/>
+      <c r="D44" s="29" t="n"/>
+      <c r="E44" s="29" t="n"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="28" t="n">
+        <v>760</v>
+      </c>
+      <c r="B45" s="29" t="n"/>
+      <c r="C45" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  4.5"  </t>
+        </is>
+      </c>
+      <c r="D45" s="31" t="inlineStr">
+        <is>
+          <t>4.5" Prod</t>
+        </is>
+      </c>
+      <c r="E45" s="29" t="n"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="28" t="inlineStr"/>
+      <c r="B46" s="29" t="n"/>
+      <c r="C46" s="36" t="inlineStr"/>
+      <c r="D46" s="29" t="n"/>
+      <c r="E46" s="29" t="n"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="28" t="n">
+        <v>800</v>
+      </c>
+      <c r="B47" s="34" t="inlineStr">
+        <is>
+          <t>Packer Shell</t>
+        </is>
+      </c>
+      <c r="C47" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  4.5"  </t>
+        </is>
+      </c>
+      <c r="D47" s="31" t="inlineStr">
+        <is>
+          <t>4.5" Prod</t>
+        </is>
+      </c>
+      <c r="E47" s="29" t="n"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="28" t="inlineStr"/>
+      <c r="B48" s="34" t="inlineStr">
+        <is>
+          <t>Packer Shell</t>
+        </is>
+      </c>
+      <c r="C48" s="36" t="inlineStr"/>
+      <c r="D48" s="29" t="n"/>
+      <c r="E48" s="29" t="n"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="28" t="n">
+        <v>840</v>
+      </c>
+      <c r="B49" s="29" t="n"/>
+      <c r="C49" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  4.5"  </t>
+        </is>
+      </c>
+      <c r="D49" s="31" t="inlineStr">
+        <is>
+          <t>4.5" Prod</t>
+        </is>
+      </c>
+      <c r="E49" s="29" t="n"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="28" t="inlineStr"/>
+      <c r="B50" s="29" t="n"/>
+      <c r="C50" s="36" t="inlineStr"/>
+      <c r="D50" s="29" t="n"/>
+      <c r="E50" s="29" t="n"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="28" t="n">
+        <v>880</v>
+      </c>
+      <c r="B51" s="29" t="n"/>
+      <c r="C51" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  4.5"  </t>
+        </is>
+      </c>
+      <c r="D51" s="31" t="inlineStr">
+        <is>
+          <t>4.5" Prod</t>
+        </is>
+      </c>
+      <c r="E51" s="29" t="n"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="28" t="inlineStr"/>
+      <c r="B52" s="29" t="n"/>
+      <c r="C52" s="36" t="inlineStr"/>
+      <c r="D52" s="29" t="n"/>
+      <c r="E52" s="29" t="n"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="28" t="n">
+        <v>920</v>
+      </c>
+      <c r="B53" s="29" t="n"/>
+      <c r="C53" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  4.5"  </t>
+        </is>
+      </c>
+      <c r="D53" s="31" t="inlineStr">
+        <is>
+          <t>4.5" Prod</t>
+        </is>
+      </c>
+      <c r="E53" s="29" t="n"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="28" t="inlineStr"/>
+      <c r="B54" s="29" t="n"/>
+      <c r="C54" s="36" t="inlineStr"/>
+      <c r="D54" s="29" t="n"/>
+      <c r="E54" s="29" t="n"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="28" t="n">
+        <v>960</v>
+      </c>
+      <c r="B55" s="29" t="n"/>
+      <c r="C55" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  4.5"  </t>
+        </is>
+      </c>
+      <c r="D55" s="31" t="inlineStr">
+        <is>
+          <t>4.5" Prod</t>
+        </is>
+      </c>
+      <c r="E55" s="29" t="n"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="28" t="inlineStr"/>
+      <c r="B56" s="29" t="n"/>
+      <c r="C56" s="36" t="inlineStr"/>
+      <c r="D56" s="29" t="n"/>
+      <c r="E56" s="29" t="n"/>
+    </row>
+    <row r="57">
+      <c r="A57" s="28" t="n">
+        <v>1000</v>
+      </c>
+      <c r="B57" s="29" t="n"/>
+      <c r="C57" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  4.5"  </t>
+        </is>
+      </c>
+      <c r="D57" s="31" t="inlineStr">
+        <is>
+          <t>4.5" Prod</t>
+        </is>
+      </c>
+      <c r="E57" s="29" t="n"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="28" t="inlineStr"/>
+      <c r="B58" s="29" t="n"/>
+      <c r="C58" s="36" t="inlineStr"/>
+      <c r="D58" s="29" t="n"/>
+      <c r="E58" s="29" t="n"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="28" t="n">
+        <v>1040</v>
+      </c>
+      <c r="B59" s="29" t="n"/>
+      <c r="C59" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  4.5"  </t>
+        </is>
+      </c>
+      <c r="D59" s="31" t="inlineStr">
+        <is>
+          <t>4.5" Prod</t>
+        </is>
+      </c>
+      <c r="E59" s="29" t="n"/>
+    </row>
+    <row r="60">
+      <c r="A60" s="28" t="inlineStr"/>
+      <c r="B60" s="29" t="n"/>
+      <c r="C60" s="36" t="inlineStr"/>
+      <c r="D60" s="29" t="n"/>
+      <c r="E60" s="29" t="n"/>
+    </row>
+    <row r="61">
+      <c r="A61" s="28" t="n">
+        <v>1080</v>
+      </c>
+      <c r="B61" s="29" t="n"/>
+      <c r="C61" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  4.5"  </t>
+        </is>
+      </c>
+      <c r="D61" s="31" t="inlineStr">
+        <is>
+          <t>4.5" Prod</t>
+        </is>
+      </c>
+      <c r="E61" s="29" t="n"/>
+    </row>
+    <row r="62">
+      <c r="A62" s="28" t="inlineStr"/>
+      <c r="B62" s="29" t="n"/>
+      <c r="C62" s="36" t="inlineStr"/>
+      <c r="D62" s="29" t="n"/>
+      <c r="E62" s="29" t="n"/>
+    </row>
+    <row r="63">
+      <c r="A63" s="28" t="n">
+        <v>1120</v>
+      </c>
+      <c r="B63" s="29" t="n"/>
+      <c r="C63" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  4.5"  </t>
+        </is>
+      </c>
+      <c r="D63" s="31" t="inlineStr">
+        <is>
+          <t>4.5" Prod</t>
+        </is>
+      </c>
+      <c r="E63" s="29" t="n"/>
+    </row>
+    <row r="64">
+      <c r="A64" s="28" t="inlineStr"/>
+      <c r="B64" s="29" t="n"/>
+      <c r="C64" s="36" t="inlineStr"/>
+      <c r="D64" s="29" t="n"/>
+      <c r="E64" s="29" t="n"/>
+    </row>
+    <row r="65">
+      <c r="A65" s="28" t="n">
+        <v>1160</v>
+      </c>
+      <c r="B65" s="29" t="n"/>
+      <c r="C65" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  4.5"  </t>
+        </is>
+      </c>
+      <c r="D65" s="31" t="inlineStr">
+        <is>
+          <t>4.5" Prod</t>
+        </is>
+      </c>
+      <c r="E65" s="29" t="n"/>
+    </row>
+    <row r="66">
+      <c r="A66" s="28" t="inlineStr"/>
+      <c r="B66" s="29" t="n"/>
+      <c r="C66" s="36" t="inlineStr"/>
+      <c r="D66" s="29" t="n"/>
+      <c r="E66" s="29" t="n"/>
+    </row>
+    <row r="67">
+      <c r="A67" s="28" t="n">
+        <v>1200</v>
+      </c>
+      <c r="B67" s="29" t="n"/>
+      <c r="C67" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  4.5"  </t>
+        </is>
+      </c>
+      <c r="D67" s="31" t="inlineStr">
+        <is>
+          <t>4.5" Prod</t>
+        </is>
+      </c>
+      <c r="E67" s="29" t="n"/>
+    </row>
+    <row r="68">
+      <c r="A68" s="28" t="inlineStr"/>
+      <c r="B68" s="29" t="n"/>
+      <c r="C68" s="36" t="inlineStr"/>
+      <c r="D68" s="29" t="n"/>
+      <c r="E68" s="29" t="n"/>
+    </row>
+    <row r="69">
+      <c r="A69" s="28" t="n">
+        <v>1240</v>
+      </c>
+      <c r="B69" s="29" t="n"/>
+      <c r="C69" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  4.5"  </t>
+        </is>
+      </c>
+      <c r="D69" s="31" t="inlineStr">
+        <is>
+          <t>4.5" Prod</t>
+        </is>
+      </c>
+      <c r="E69" s="29" t="n"/>
+    </row>
+    <row r="70">
+      <c r="A70" s="28" t="inlineStr"/>
+      <c r="B70" s="29" t="n"/>
+      <c r="C70" s="36" t="inlineStr"/>
+      <c r="D70" s="29" t="n"/>
+      <c r="E70" s="29" t="n"/>
+    </row>
+    <row r="71">
+      <c r="A71" s="28" t="n">
+        <v>1280</v>
+      </c>
+      <c r="B71" s="29" t="n"/>
+      <c r="C71" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  4.5"  </t>
+        </is>
+      </c>
+      <c r="D71" s="31" t="inlineStr">
+        <is>
+          <t>4.5" Prod</t>
+        </is>
+      </c>
+      <c r="E71" s="29" t="n"/>
+    </row>
+    <row r="72">
+      <c r="A72" s="28" t="inlineStr"/>
+      <c r="B72" s="29" t="n"/>
+      <c r="C72" s="36" t="inlineStr"/>
+      <c r="D72" s="29" t="n"/>
+      <c r="E72" s="29" t="n"/>
+    </row>
+    <row r="73">
+      <c r="A73" s="28" t="n">
+        <v>1320</v>
+      </c>
+      <c r="B73" s="29" t="n"/>
+      <c r="C73" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  4.5"  </t>
+        </is>
+      </c>
+      <c r="D73" s="31" t="inlineStr">
+        <is>
+          <t>4.5" Prod</t>
+        </is>
+      </c>
+      <c r="E73" s="29" t="n"/>
+    </row>
+    <row r="74">
+      <c r="A74" s="28" t="inlineStr"/>
+      <c r="B74" s="29" t="n"/>
+      <c r="C74" s="36" t="inlineStr"/>
+      <c r="D74" s="29" t="n"/>
+      <c r="E74" s="29" t="n"/>
+    </row>
+    <row r="75">
+      <c r="A75" s="28" t="n">
+        <v>1360</v>
+      </c>
+      <c r="B75" s="29" t="n"/>
+      <c r="C75" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  4.5"  </t>
+        </is>
+      </c>
+      <c r="D75" s="31" t="inlineStr">
+        <is>
+          <t>4.5" Prod</t>
+        </is>
+      </c>
+      <c r="E75" s="29" t="n"/>
+    </row>
+    <row r="76">
+      <c r="A76" s="28" t="inlineStr"/>
+      <c r="B76" s="29" t="n"/>
+      <c r="C76" s="36" t="inlineStr"/>
+      <c r="D76" s="29" t="n"/>
+      <c r="E76" s="29" t="n"/>
+    </row>
+    <row r="77">
+      <c r="A77" s="28" t="n">
+        <v>1400</v>
+      </c>
+      <c r="B77" s="29" t="n"/>
+      <c r="C77" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  4.5"  </t>
+        </is>
+      </c>
+      <c r="D77" s="31" t="inlineStr">
+        <is>
+          <t>4.5" Prod</t>
+        </is>
+      </c>
+      <c r="E77" s="29" t="n"/>
+    </row>
+    <row r="78">
+      <c r="A78" s="28" t="inlineStr"/>
+      <c r="B78" s="29" t="n"/>
+      <c r="C78" s="36" t="inlineStr"/>
+      <c r="D78" s="29" t="n"/>
+      <c r="E78" s="29" t="n"/>
+    </row>
+    <row r="79">
+      <c r="A79" s="28" t="n">
+        <v>1440</v>
+      </c>
+      <c r="B79" s="29" t="n"/>
+      <c r="C79" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  4.5"  </t>
+        </is>
+      </c>
+      <c r="D79" s="31" t="inlineStr">
+        <is>
+          <t>4.5" Prod</t>
+        </is>
+      </c>
+      <c r="E79" s="29" t="n"/>
+    </row>
+    <row r="80">
+      <c r="A80" s="28" t="inlineStr"/>
+      <c r="B80" s="29" t="n"/>
+      <c r="C80" s="36" t="inlineStr"/>
+      <c r="D80" s="29" t="n"/>
+      <c r="E80" s="29" t="n"/>
+    </row>
+    <row r="81">
+      <c r="A81" s="28" t="n">
+        <v>1480</v>
+      </c>
+      <c r="B81" s="29" t="n"/>
+      <c r="C81" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  4.5"  </t>
+        </is>
+      </c>
+      <c r="D81" s="31" t="inlineStr">
+        <is>
+          <t>4.5" Prod</t>
+        </is>
+      </c>
+      <c r="E81" s="29" t="n"/>
+    </row>
+    <row r="82">
+      <c r="A82" s="28" t="inlineStr"/>
+      <c r="B82" s="29" t="n"/>
+      <c r="C82" s="36" t="inlineStr"/>
+      <c r="D82" s="29" t="n"/>
+      <c r="E82" s="29" t="n"/>
+    </row>
+    <row r="83">
+      <c r="A83" s="28" t="n">
+        <v>1520</v>
+      </c>
+      <c r="B83" s="29" t="n"/>
+      <c r="C83" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  4.5"  </t>
+        </is>
+      </c>
+      <c r="D83" s="31" t="inlineStr">
+        <is>
+          <t>4.5" Prod</t>
+        </is>
+      </c>
+      <c r="E83" s="29" t="n"/>
+    </row>
+    <row r="84">
+      <c r="A84" s="28" t="inlineStr"/>
+      <c r="B84" s="29" t="n"/>
+      <c r="C84" s="36" t="inlineStr"/>
+      <c r="D84" s="29" t="n"/>
+      <c r="E84" s="29" t="n"/>
+    </row>
+    <row r="85">
+      <c r="A85" s="28" t="n">
+        <v>1560</v>
+      </c>
+      <c r="B85" s="29" t="n"/>
+      <c r="C85" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  4.5"  </t>
+        </is>
+      </c>
+      <c r="D85" s="31" t="inlineStr">
+        <is>
+          <t>4.5" Prod</t>
+        </is>
+      </c>
+      <c r="E85" s="29" t="n"/>
+    </row>
+    <row r="86">
+      <c r="A86" s="28" t="inlineStr"/>
+      <c r="B86" s="29" t="n"/>
+      <c r="C86" s="36" t="inlineStr"/>
+      <c r="D86" s="29" t="n"/>
+      <c r="E86" s="29" t="n"/>
+    </row>
+    <row r="87">
+      <c r="A87" s="28" t="n">
+        <v>1600</v>
+      </c>
+      <c r="B87" s="29" t="n"/>
+      <c r="C87" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  4.5"  </t>
+        </is>
+      </c>
+      <c r="D87" s="31" t="inlineStr">
+        <is>
+          <t>4.5" Prod</t>
+        </is>
+      </c>
+      <c r="E87" s="29" t="n"/>
+    </row>
+    <row r="88">
+      <c r="A88" s="28" t="inlineStr"/>
+      <c r="B88" s="29" t="n"/>
+      <c r="C88" s="36" t="inlineStr"/>
+      <c r="D88" s="29" t="n"/>
+      <c r="E88" s="29" t="n"/>
+    </row>
+    <row r="89">
+      <c r="A89" s="28" t="n">
+        <v>1640</v>
+      </c>
+      <c r="B89" s="29" t="n"/>
+      <c r="C89" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  4.5"  </t>
+        </is>
+      </c>
+      <c r="D89" s="31" t="inlineStr">
+        <is>
+          <t>4.5" Prod</t>
+        </is>
+      </c>
+      <c r="E89" s="29" t="n"/>
+    </row>
+    <row r="90">
+      <c r="A90" s="28" t="inlineStr"/>
+      <c r="B90" s="29" t="n"/>
+      <c r="C90" s="36" t="inlineStr"/>
+      <c r="D90" s="29" t="n"/>
+      <c r="E90" s="29" t="n"/>
+    </row>
+    <row r="91">
+      <c r="A91" s="28" t="n">
+        <v>1680</v>
+      </c>
+      <c r="B91" s="29" t="n"/>
+      <c r="C91" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  4.5"  </t>
+        </is>
+      </c>
+      <c r="D91" s="31" t="inlineStr">
+        <is>
+          <t>4.5" Prod</t>
+        </is>
+      </c>
+      <c r="E91" s="29" t="n"/>
+    </row>
+    <row r="92">
+      <c r="A92" s="28" t="inlineStr"/>
+      <c r="B92" s="29" t="n"/>
+      <c r="C92" s="36" t="inlineStr"/>
+      <c r="D92" s="29" t="n"/>
+      <c r="E92" s="29" t="n"/>
+    </row>
+    <row r="93">
+      <c r="A93" s="28" t="n">
+        <v>1720</v>
+      </c>
+      <c r="B93" s="29" t="n"/>
+      <c r="C93" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  4.5"  </t>
+        </is>
+      </c>
+      <c r="D93" s="31" t="inlineStr">
+        <is>
+          <t>4.5" Prod</t>
+        </is>
+      </c>
+      <c r="E93" s="29" t="n"/>
+    </row>
+    <row r="94">
+      <c r="A94" s="28" t="inlineStr"/>
+      <c r="B94" s="29" t="n"/>
+      <c r="C94" s="36" t="inlineStr"/>
+      <c r="D94" s="29" t="n"/>
+      <c r="E94" s="29" t="n"/>
+    </row>
+    <row r="95">
+      <c r="A95" s="28" t="n">
+        <v>1760</v>
+      </c>
+      <c r="B95" s="29" t="n"/>
+      <c r="C95" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  4.5"  </t>
+        </is>
+      </c>
+      <c r="D95" s="31" t="inlineStr">
+        <is>
+          <t>4.5" Prod</t>
+        </is>
+      </c>
+      <c r="E95" s="29" t="n"/>
+    </row>
+    <row r="96">
+      <c r="A96" s="28" t="inlineStr"/>
+      <c r="B96" s="29" t="n"/>
+      <c r="C96" s="36" t="inlineStr"/>
+      <c r="D96" s="29" t="n"/>
+      <c r="E96" s="29" t="n"/>
+    </row>
+    <row r="97">
+      <c r="A97" s="28" t="n">
+        <v>1800</v>
+      </c>
+      <c r="B97" s="29" t="n"/>
+      <c r="C97" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  4.5"  </t>
+        </is>
+      </c>
+      <c r="D97" s="31" t="inlineStr">
+        <is>
+          <t>4.5" Prod</t>
+        </is>
+      </c>
+      <c r="E97" s="29" t="n"/>
+    </row>
+    <row r="98">
+      <c r="A98" s="28" t="inlineStr"/>
+      <c r="B98" s="29" t="n"/>
+      <c r="C98" s="36" t="inlineStr"/>
+      <c r="D98" s="29" t="n"/>
+      <c r="E98" s="29" t="n"/>
+    </row>
+    <row r="99">
+      <c r="A99" s="28" t="n">
+        <v>1840</v>
+      </c>
+      <c r="B99" s="29" t="n"/>
+      <c r="C99" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  4.5"  </t>
+        </is>
+      </c>
+      <c r="D99" s="31" t="inlineStr">
+        <is>
+          <t>4.5" Prod</t>
+        </is>
+      </c>
+      <c r="E99" s="29" t="n"/>
+    </row>
+    <row r="100">
+      <c r="A100" s="28" t="inlineStr"/>
+      <c r="B100" s="29" t="n"/>
+      <c r="C100" s="36" t="inlineStr"/>
+      <c r="D100" s="29" t="n"/>
+      <c r="E100" s="29" t="n"/>
+    </row>
+    <row r="101">
+      <c r="A101" s="28" t="n">
+        <v>1880</v>
+      </c>
+      <c r="B101" s="29" t="n"/>
+      <c r="C101" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  4.5"  </t>
+        </is>
+      </c>
+      <c r="D101" s="31" t="inlineStr">
+        <is>
+          <t>4.5" Prod</t>
+        </is>
+      </c>
+      <c r="E101" s="29" t="n"/>
+    </row>
+    <row r="102">
+      <c r="A102" s="28" t="inlineStr"/>
+      <c r="B102" s="29" t="n"/>
+      <c r="C102" s="36" t="inlineStr"/>
+      <c r="D102" s="29" t="n"/>
+      <c r="E102" s="29" t="n"/>
+    </row>
+    <row r="103">
+      <c r="A103" s="28" t="n">
+        <v>1920</v>
+      </c>
+      <c r="B103" s="29" t="n"/>
+      <c r="C103" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  4.5"  </t>
+        </is>
+      </c>
+      <c r="D103" s="31" t="inlineStr">
+        <is>
+          <t>4.5" Prod</t>
+        </is>
+      </c>
+      <c r="E103" s="29" t="n"/>
+    </row>
+    <row r="104">
+      <c r="A104" s="28" t="inlineStr"/>
+      <c r="B104" s="29" t="n"/>
+      <c r="C104" s="36" t="inlineStr"/>
+      <c r="D104" s="29" t="n"/>
+      <c r="E104" s="29" t="n"/>
+    </row>
+    <row r="105">
+      <c r="A105" s="28" t="n">
+        <v>1960</v>
+      </c>
+      <c r="B105" s="37" t="inlineStr">
+        <is>
+          <t>Trenton Limestone</t>
+        </is>
+      </c>
+      <c r="C105" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  4.5"  </t>
+        </is>
+      </c>
+      <c r="D105" s="31" t="inlineStr">
+        <is>
+          <t>4.5" Prod</t>
+        </is>
+      </c>
+      <c r="E105" s="29" t="n"/>
+    </row>
+    <row r="106">
+      <c r="A106" s="28" t="inlineStr"/>
+      <c r="B106" s="37" t="inlineStr">
+        <is>
+          <t>Trenton Limestone</t>
+        </is>
+      </c>
+      <c r="C106" s="36" t="inlineStr"/>
+      <c r="D106" s="29" t="n"/>
+      <c r="E106" s="29" t="n"/>
+    </row>
+    <row r="107">
+      <c r="A107" s="28" t="n">
+        <v>2000</v>
+      </c>
+      <c r="B107" s="37" t="inlineStr"/>
+      <c r="C107" s="38" t="inlineStr"/>
+      <c r="D107" s="29" t="n"/>
+      <c r="E107" s="29" t="n"/>
+    </row>
+    <row r="108">
+      <c r="A108" s="28" t="inlineStr"/>
+      <c r="B108" s="37" t="inlineStr"/>
+      <c r="C108" s="38" t="inlineStr"/>
+      <c r="D108" s="29" t="n"/>
+      <c r="E108" s="29" t="n"/>
+    </row>
+    <row r="109">
+      <c r="A109" s="28" t="n">
+        <v>2040</v>
+      </c>
+      <c r="B109" s="37" t="inlineStr">
+        <is>
+          <t>Trenton Limestone</t>
+        </is>
+      </c>
+      <c r="C109" s="38" t="inlineStr">
         <is>
           <t xml:space="preserve">  ∅  </t>
         </is>
       </c>
-      <c r="D43" s="26" t="n"/>
-      <c r="E43" s="26" t="n"/>
-    </row>
-    <row r="44">
-      <c r="A44" s="25" t="inlineStr"/>
-      <c r="B44" s="32" t="inlineStr"/>
-      <c r="C44" s="33" t="inlineStr"/>
-      <c r="D44" s="26" t="n"/>
-      <c r="E44" s="26" t="n"/>
-    </row>
-    <row r="45">
-      <c r="A45" s="25" t="n">
-        <v>380</v>
-      </c>
-      <c r="B45" s="32" t="inlineStr"/>
-      <c r="C45" s="33" t="inlineStr"/>
-      <c r="D45" s="26" t="n"/>
-      <c r="E45" s="26" t="n"/>
-    </row>
-    <row r="46">
-      <c r="A46" s="25" t="inlineStr"/>
-      <c r="B46" s="32" t="inlineStr">
-        <is>
-          <t>Big Lime</t>
-        </is>
-      </c>
-      <c r="C46" s="33" t="inlineStr">
+      <c r="D109" s="29" t="n"/>
+      <c r="E109" s="32" t="inlineStr">
+        <is>
+          <t>Hole: 6" Open Hole (below production casing) to total depth 2458'</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="28" t="inlineStr"/>
+      <c r="B110" s="37" t="inlineStr"/>
+      <c r="C110" s="38" t="inlineStr"/>
+      <c r="D110" s="29" t="n"/>
+      <c r="E110" s="29" t="n"/>
+    </row>
+    <row r="111">
+      <c r="A111" s="28" t="n">
+        <v>2080</v>
+      </c>
+      <c r="B111" s="37" t="inlineStr"/>
+      <c r="C111" s="38" t="inlineStr"/>
+      <c r="D111" s="29" t="n"/>
+      <c r="E111" s="29" t="n"/>
+    </row>
+    <row r="112">
+      <c r="A112" s="28" t="inlineStr"/>
+      <c r="B112" s="37" t="inlineStr">
+        <is>
+          <t>Trenton Limestone</t>
+        </is>
+      </c>
+      <c r="C112" s="38" t="inlineStr">
         <is>
           <t xml:space="preserve">  ∅  </t>
         </is>
       </c>
-      <c r="D46" s="26" t="n"/>
-      <c r="E46" s="26" t="n"/>
-    </row>
-    <row r="47">
-      <c r="A47" s="25" t="n">
-        <v>400</v>
-      </c>
-      <c r="B47" s="32" t="inlineStr"/>
-      <c r="C47" s="33" t="inlineStr"/>
-      <c r="D47" s="26" t="n"/>
-      <c r="E47" s="26" t="n"/>
-    </row>
-    <row r="48">
-      <c r="A48" s="3" t="inlineStr">
-        <is>
-          <t>— Deeper sections (Trenton 1944'– , Black River to 2458') per original Excel / add data rows above and extend schematic —</t>
-        </is>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" s="34" t="inlineStr">
+      <c r="D112" s="29" t="n"/>
+      <c r="E112" s="29" t="n"/>
+    </row>
+    <row r="113">
+      <c r="A113" s="28" t="n">
+        <v>2120</v>
+      </c>
+      <c r="B113" s="35" t="inlineStr">
+        <is>
+          <t>Black River Group</t>
+        </is>
+      </c>
+      <c r="C113" s="38" t="inlineStr"/>
+      <c r="D113" s="29" t="n"/>
+      <c r="E113" s="29" t="n"/>
+    </row>
+    <row r="114">
+      <c r="A114" s="28" t="inlineStr"/>
+      <c r="B114" s="35" t="inlineStr">
+        <is>
+          <t>Black River Group</t>
+        </is>
+      </c>
+      <c r="C114" s="38" t="inlineStr"/>
+      <c r="D114" s="29" t="n"/>
+      <c r="E114" s="29" t="n"/>
+    </row>
+    <row r="115">
+      <c r="A115" s="28" t="n">
+        <v>2160</v>
+      </c>
+      <c r="B115" s="35" t="inlineStr">
+        <is>
+          <t>Black River Group</t>
+        </is>
+      </c>
+      <c r="C115" s="38" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ∅  </t>
+        </is>
+      </c>
+      <c r="D115" s="29" t="n"/>
+      <c r="E115" s="29" t="n"/>
+    </row>
+    <row r="116">
+      <c r="A116" s="28" t="inlineStr"/>
+      <c r="B116" s="35" t="inlineStr"/>
+      <c r="C116" s="38" t="inlineStr"/>
+      <c r="D116" s="29" t="n"/>
+      <c r="E116" s="29" t="n"/>
+    </row>
+    <row r="117">
+      <c r="A117" s="28" t="n">
+        <v>2200</v>
+      </c>
+      <c r="B117" s="35" t="inlineStr"/>
+      <c r="C117" s="38" t="inlineStr"/>
+      <c r="D117" s="29" t="n"/>
+      <c r="E117" s="29" t="n"/>
+    </row>
+    <row r="118">
+      <c r="A118" s="28" t="inlineStr"/>
+      <c r="B118" s="35" t="inlineStr">
+        <is>
+          <t>Black River Group</t>
+        </is>
+      </c>
+      <c r="C118" s="38" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ∅  </t>
+        </is>
+      </c>
+      <c r="D118" s="29" t="n"/>
+      <c r="E118" s="29" t="n"/>
+    </row>
+    <row r="119">
+      <c r="A119" s="28" t="n">
+        <v>2240</v>
+      </c>
+      <c r="B119" s="35" t="inlineStr"/>
+      <c r="C119" s="38" t="inlineStr"/>
+      <c r="D119" s="29" t="n"/>
+      <c r="E119" s="29" t="n"/>
+    </row>
+    <row r="120">
+      <c r="A120" s="28" t="inlineStr"/>
+      <c r="B120" s="35" t="inlineStr"/>
+      <c r="C120" s="38" t="inlineStr"/>
+      <c r="D120" s="29" t="n"/>
+      <c r="E120" s="29" t="n"/>
+    </row>
+    <row r="121">
+      <c r="A121" s="28" t="n">
+        <v>2280</v>
+      </c>
+      <c r="B121" s="35" t="inlineStr">
+        <is>
+          <t>Black River Group</t>
+        </is>
+      </c>
+      <c r="C121" s="38" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ∅  </t>
+        </is>
+      </c>
+      <c r="D121" s="29" t="n"/>
+      <c r="E121" s="29" t="n"/>
+    </row>
+    <row r="122">
+      <c r="A122" s="28" t="inlineStr"/>
+      <c r="B122" s="35" t="inlineStr"/>
+      <c r="C122" s="38" t="inlineStr"/>
+      <c r="D122" s="29" t="n"/>
+      <c r="E122" s="29" t="n"/>
+    </row>
+    <row r="123">
+      <c r="A123" s="28" t="n">
+        <v>2320</v>
+      </c>
+      <c r="B123" s="35" t="inlineStr"/>
+      <c r="C123" s="38" t="inlineStr"/>
+      <c r="D123" s="29" t="n"/>
+      <c r="E123" s="29" t="n"/>
+    </row>
+    <row r="124">
+      <c r="A124" s="28" t="inlineStr"/>
+      <c r="B124" s="35" t="inlineStr">
+        <is>
+          <t>Black River Group</t>
+        </is>
+      </c>
+      <c r="C124" s="38" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ∅  </t>
+        </is>
+      </c>
+      <c r="D124" s="29" t="n"/>
+      <c r="E124" s="29" t="n"/>
+    </row>
+    <row r="125">
+      <c r="A125" s="28" t="n">
+        <v>2360</v>
+      </c>
+      <c r="B125" s="35" t="inlineStr"/>
+      <c r="C125" s="38" t="inlineStr"/>
+      <c r="D125" s="29" t="n"/>
+      <c r="E125" s="29" t="n"/>
+    </row>
+    <row r="126">
+      <c r="A126" s="28" t="inlineStr"/>
+      <c r="B126" s="35" t="inlineStr"/>
+      <c r="C126" s="38" t="inlineStr"/>
+      <c r="D126" s="29" t="n"/>
+      <c r="E126" s="29" t="n"/>
+    </row>
+    <row r="127">
+      <c r="A127" s="28" t="n">
+        <v>2400</v>
+      </c>
+      <c r="B127" s="35" t="inlineStr">
+        <is>
+          <t>Black River Group</t>
+        </is>
+      </c>
+      <c r="C127" s="38" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ∅  </t>
+        </is>
+      </c>
+      <c r="D127" s="29" t="n"/>
+      <c r="E127" s="29" t="n"/>
+    </row>
+    <row r="128">
+      <c r="A128" s="28" t="inlineStr"/>
+      <c r="B128" s="35" t="inlineStr"/>
+      <c r="C128" s="38" t="inlineStr"/>
+      <c r="D128" s="29" t="n"/>
+      <c r="E128" s="29" t="n"/>
+    </row>
+    <row r="129">
+      <c r="A129" s="28" t="n">
+        <v>2440</v>
+      </c>
+      <c r="B129" s="35" t="inlineStr"/>
+      <c r="C129" s="38" t="inlineStr"/>
+      <c r="D129" s="29" t="n"/>
+      <c r="E129" s="29" t="n"/>
+    </row>
+    <row r="130">
+      <c r="A130" s="28" t="inlineStr"/>
+      <c r="B130" s="29" t="n"/>
+      <c r="C130" s="38" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ∅  </t>
+        </is>
+      </c>
+      <c r="D130" s="29" t="n"/>
+      <c r="E130" s="29" t="n"/>
+    </row>
+    <row r="131">
+      <c r="A131" s="28" t="n">
+        <v>2480</v>
+      </c>
+      <c r="B131" s="29" t="n"/>
+      <c r="C131" s="38" t="inlineStr"/>
+      <c r="D131" s="29" t="n"/>
+      <c r="E131" s="29" t="n"/>
+    </row>
+    <row r="132">
+      <c r="A132" s="28" t="inlineStr"/>
+      <c r="B132" s="29" t="n"/>
+      <c r="C132" s="38" t="inlineStr"/>
+      <c r="D132" s="29" t="n"/>
+      <c r="E132" s="29" t="n"/>
+    </row>
+    <row r="133">
+      <c r="A133" s="3" t="inlineStr">
+        <is>
+          <t>— Total vertical depth represented down to Black River Group (2458') —</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" s="39" t="inlineStr">
         <is>
           <t>TOPOLOGICAL VERIFICATION (welly_db_4budZ harness)</t>
         </is>
       </c>
     </row>
-    <row r="51">
-      <c r="A51" s="35" t="inlineStr">
-        <is>
-          <t>Δλ₁ = +0.0801 (positive coherence harvest)  •  Holonomy: trivial  •  lambda_1 ≈ 1.001  •  2 nodes (Conductor + Surface)  •  Evidence: K_S_evidence_*.json in artifacts/</t>
+    <row r="136">
+      <c r="A136" s="40" t="inlineStr">
+        <is>
+          <t>Δλ₁ = +0.0800 (positive coherence harvest)  •  Holonomy: trivial  •  lambda_1 ≈ 1.000  •  3 nodes (Conductor + Surface + Production)  •  Evidence: K_S_evidence_*.json in artifacts/</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="5">
     <mergeCell ref="A2:F2"/>
-    <mergeCell ref="A50:E50"/>
-    <mergeCell ref="A48:E48"/>
     <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A51:E51"/>
+    <mergeCell ref="A133:F133"/>
+    <mergeCell ref="A136:F136"/>
+    <mergeCell ref="A135:F135"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>